<commit_message>
Actualización automática desde sistema web
</commit_message>
<xml_diff>
--- a/znomatriz2026.xlsx
+++ b/znomatriz2026.xlsx
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>NOROCCIDENTE</v>
+        <v>NO</v>
       </c>
       <c r="C2" t="str">
         <v>Chamanga</v>
@@ -454,7 +454,7 @@
         <v>ZNO_REE_DPA.CHAMANGA_BK1_2</v>
       </c>
       <c r="F2" t="str">
-        <v>PB1</v>
+        <v>PB</v>
       </c>
       <c r="G2" t="str">
         <v xml:space="preserve"> CHAMANGA</v>

</xml_diff>